<commit_message>
criação da pasta trello
</commit_message>
<xml_diff>
--- a/relatorio/base.xlsx
+++ b/relatorio/base.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\Produção\Etiquetas\Nova pasta\relatorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Produção\Etiquetas\Nova pasta\relatorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90C666A-27C5-4831-A5D5-F53F12275F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3087,9 +3086,6 @@
     <t>7899884535851</t>
   </si>
   <si>
-    <t>CHAVETA DE DESTRAVAMENTO PIVÔ EX</t>
-  </si>
-  <si>
     <t>7899884536353</t>
   </si>
   <si>
@@ -3319,12 +3315,15 @@
   </si>
   <si>
     <t>ROLAMENTO DO MANCAL DA TESTEIRA DO 200/300</t>
+  </si>
+  <si>
+    <t>PINO DE DESTRAVAMENTO MANUAL PIVOTANTE EX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3404,7 +3403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3418,6 +3417,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3698,7 +3700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E577"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -12316,11 +12318,11 @@
       <c r="A509">
         <v>2010349</v>
       </c>
-      <c r="B509" t="s">
+      <c r="B509" s="6" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C509" s="3" t="s">
         <v>1013</v>
-      </c>
-      <c r="C509" s="3" t="s">
-        <v>1014</v>
       </c>
       <c r="D509" t="s">
         <v>7</v>
@@ -12334,10 +12336,10 @@
         <v>2010495</v>
       </c>
       <c r="B510" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C510" s="3" t="s">
         <v>1015</v>
-      </c>
-      <c r="C510" s="3" t="s">
-        <v>1016</v>
       </c>
       <c r="D510" t="s">
         <v>7</v>
@@ -12351,10 +12353,10 @@
         <v>2010526</v>
       </c>
       <c r="B511" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C511" s="3" t="s">
         <v>1017</v>
-      </c>
-      <c r="C511" s="3" t="s">
-        <v>1018</v>
       </c>
       <c r="D511" t="s">
         <v>7</v>
@@ -12368,10 +12370,10 @@
         <v>2010373</v>
       </c>
       <c r="B512" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C512" s="3" t="s">
         <v>1019</v>
-      </c>
-      <c r="C512" s="3" t="s">
-        <v>1020</v>
       </c>
       <c r="D512" t="s">
         <v>7</v>
@@ -12385,10 +12387,10 @@
         <v>2030041</v>
       </c>
       <c r="B513" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C513" s="3" t="s">
         <v>1021</v>
-      </c>
-      <c r="C513" s="3" t="s">
-        <v>1022</v>
       </c>
       <c r="D513" t="s">
         <v>7</v>
@@ -12402,10 +12404,10 @@
         <v>2030050</v>
       </c>
       <c r="B514" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C514" s="3" t="s">
         <v>1023</v>
-      </c>
-      <c r="C514" s="3" t="s">
-        <v>1024</v>
       </c>
       <c r="D514" t="s">
         <v>7</v>
@@ -12419,10 +12421,10 @@
         <v>2001156</v>
       </c>
       <c r="B515" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C515" s="3" t="s">
         <v>1025</v>
-      </c>
-      <c r="C515" s="3" t="s">
-        <v>1026</v>
       </c>
       <c r="D515" t="s">
         <v>7</v>
@@ -12436,10 +12438,10 @@
         <v>2030040</v>
       </c>
       <c r="B516" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C516" s="3" t="s">
         <v>1027</v>
-      </c>
-      <c r="C516" s="3" t="s">
-        <v>1028</v>
       </c>
       <c r="D516" t="s">
         <v>7</v>
@@ -12453,10 +12455,10 @@
         <v>2030096</v>
       </c>
       <c r="B517" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C517" s="3" t="s">
         <v>1029</v>
-      </c>
-      <c r="C517" s="3" t="s">
-        <v>1030</v>
       </c>
       <c r="D517" t="s">
         <v>7</v>
@@ -12470,7 +12472,7 @@
         <v>1015659</v>
       </c>
       <c r="B518" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="C518" s="3">
         <v>7899884560952</v>
@@ -12481,7 +12483,7 @@
         <v>2010372</v>
       </c>
       <c r="B519" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="C519" s="3">
         <v>7899884536834</v>
@@ -12492,7 +12494,7 @@
         <v>1015613</v>
       </c>
       <c r="B520" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="C520" s="3">
         <v>7899884551905</v>
@@ -12503,7 +12505,7 @@
         <v>1015541</v>
       </c>
       <c r="B521" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="C521" s="3">
         <v>7899884527443</v>
@@ -12514,7 +12516,7 @@
         <v>1015548</v>
       </c>
       <c r="B522" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="C522" s="3">
         <v>7899884531105</v>
@@ -12525,7 +12527,7 @@
         <v>1015553</v>
       </c>
       <c r="B523" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="C523" s="3">
         <v>7899884531624</v>
@@ -12534,7 +12536,7 @@
         <v>7</v>
       </c>
       <c r="E523" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="524" spans="1:5" x14ac:dyDescent="0.25">
@@ -12542,7 +12544,7 @@
         <v>1015616</v>
       </c>
       <c r="B524" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="C524" s="3">
         <v>7899884552957</v>
@@ -12553,7 +12555,7 @@
         <v>1015544</v>
       </c>
       <c r="B525" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="C525" s="3">
         <v>7899884527825</v>
@@ -12564,7 +12566,7 @@
         <v>1015543</v>
       </c>
       <c r="B526" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="C526" s="3">
         <v>7899884527818</v>
@@ -12575,7 +12577,7 @@
         <v>2030112</v>
       </c>
       <c r="B527" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="C527" s="3">
         <v>7899884562031</v>
@@ -12586,7 +12588,7 @@
         <v>1015574</v>
       </c>
       <c r="B528" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="C528" s="3">
         <v>7899884535455</v>
@@ -12608,7 +12610,7 @@
         <v>2010527</v>
       </c>
       <c r="B530" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="C530" s="3">
         <v>7899884561980</v>
@@ -12619,7 +12621,7 @@
         <v>2010528</v>
       </c>
       <c r="B531" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="C531" s="3">
         <v>7899884561997</v>
@@ -12630,7 +12632,7 @@
         <v>2010529</v>
       </c>
       <c r="B532" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="C532" s="3">
         <v>7899884562000</v>
@@ -12641,7 +12643,7 @@
         <v>2010099</v>
       </c>
       <c r="B533" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="C533" s="3">
         <v>7899884562062</v>
@@ -12652,7 +12654,7 @@
         <v>1013510</v>
       </c>
       <c r="B534" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="C534" s="3">
         <v>7899884546000</v>
@@ -12661,7 +12663,7 @@
         <v>7</v>
       </c>
       <c r="E534" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="535" spans="1:5" x14ac:dyDescent="0.25">
@@ -12669,7 +12671,7 @@
         <v>1013507</v>
       </c>
       <c r="B535" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="C535" s="3">
         <v>7899884543955</v>
@@ -12680,7 +12682,7 @@
         <v>1110356</v>
       </c>
       <c r="B536" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="C536" s="3">
         <v>7899884533277</v>
@@ -12689,7 +12691,7 @@
         <v>258</v>
       </c>
       <c r="E536" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="537" spans="1:5" x14ac:dyDescent="0.25">
@@ -12697,7 +12699,7 @@
         <v>1015538</v>
       </c>
       <c r="B537" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="C537" s="3">
         <v>7899884527030</v>
@@ -12706,7 +12708,7 @@
         <v>258</v>
       </c>
       <c r="E537" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.25">
@@ -12714,7 +12716,7 @@
         <v>1015549</v>
       </c>
       <c r="B538" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="C538" s="3">
         <v>7892562053029</v>
@@ -12723,7 +12725,7 @@
         <v>258</v>
       </c>
       <c r="E538" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="539" spans="1:5" x14ac:dyDescent="0.25">
@@ -12731,7 +12733,7 @@
         <v>2030113</v>
       </c>
       <c r="B539" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="C539" s="3">
         <v>7899884562086</v>
@@ -12742,7 +12744,7 @@
         <v>2010535</v>
       </c>
       <c r="B540" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="C540" s="3">
         <v>7899884562543</v>
@@ -12753,7 +12755,7 @@
         <v>2010534</v>
       </c>
       <c r="B541" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="C541" s="3">
         <v>7899884562536</v>
@@ -12764,7 +12766,7 @@
         <v>2010536</v>
       </c>
       <c r="B542" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="C542" s="3">
         <v>7899884562550</v>
@@ -12775,7 +12777,7 @@
         <v>2010538</v>
       </c>
       <c r="B543" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="C543" s="5">
         <v>7899884562581</v>
@@ -12797,7 +12799,7 @@
         <v>1015661</v>
       </c>
       <c r="B545" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="C545" s="3">
         <v>7899884562598</v>
@@ -12808,7 +12810,7 @@
         <v>1015537</v>
       </c>
       <c r="B546" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="C546" s="3">
         <v>7899884527023</v>
@@ -12819,7 +12821,7 @@
         <v>2010532</v>
       </c>
       <c r="B547" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="C547" s="3">
         <v>7899884562246</v>
@@ -12827,7 +12829,7 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B548" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
@@ -12835,7 +12837,7 @@
         <v>1015615</v>
       </c>
       <c r="B549" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="C549" s="3">
         <v>7899884552629</v>
@@ -12846,7 +12848,7 @@
         <v>1015555</v>
       </c>
       <c r="B550" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="C550" s="3">
         <v>7899884531648</v>
@@ -12857,7 +12859,7 @@
         <v>1015618</v>
       </c>
       <c r="B551" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="C551" s="3">
         <v>7899884552971</v>
@@ -12868,7 +12870,7 @@
         <v>2003062</v>
       </c>
       <c r="B552" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="C552" s="3">
         <v>7899884558423</v>
@@ -12879,7 +12881,7 @@
         <v>2014024</v>
       </c>
       <c r="B553" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C553" s="3">
         <v>7899884560808</v>
@@ -12890,7 +12892,7 @@
         <v>2014025</v>
       </c>
       <c r="B554" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="C554" s="3">
         <v>7899884560815</v>
@@ -12901,7 +12903,7 @@
         <v>1015032</v>
       </c>
       <c r="B555" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="C555" s="3">
         <v>7899884553732</v>
@@ -12912,7 +12914,7 @@
         <v>1015559</v>
       </c>
       <c r="B556" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="C556" s="3">
         <v>7899884532089</v>
@@ -12923,7 +12925,7 @@
         <v>1015640</v>
       </c>
       <c r="B557" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="C557" s="3">
         <v>7899884559024</v>
@@ -12934,7 +12936,7 @@
         <v>1015626</v>
       </c>
       <c r="B558" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C558" s="3">
         <v>7899884553640</v>
@@ -12945,7 +12947,7 @@
         <v>1015636</v>
       </c>
       <c r="B559" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="C559" s="3">
         <v>7899884558980</v>
@@ -12956,7 +12958,7 @@
         <v>2010454</v>
       </c>
       <c r="B560" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="C560" s="3">
         <v>7899884557303</v>
@@ -12967,7 +12969,7 @@
         <v>2004028</v>
       </c>
       <c r="B561" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="C561" s="3">
         <v>7899884534717</v>
@@ -12978,7 +12980,7 @@
         <v>1015648</v>
       </c>
       <c r="B562" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="C562" s="3">
         <v>7899884557259</v>
@@ -12989,7 +12991,7 @@
         <v>1015580</v>
       </c>
       <c r="B563" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="C563" s="3">
         <v>7899884539170</v>
@@ -13000,7 +13002,7 @@
         <v>1110351</v>
       </c>
       <c r="B564" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="C564" s="3">
         <v>7899884532737</v>
@@ -13011,7 +13013,7 @@
         <v>1015662</v>
       </c>
       <c r="B565" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C565" s="3">
         <v>7899884563397</v>
@@ -13022,7 +13024,7 @@
         <v>2010157</v>
       </c>
       <c r="B566" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C566" s="3">
         <v>7899884563397</v>
@@ -13033,7 +13035,7 @@
         <v>1015569</v>
       </c>
       <c r="B567" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="C567" s="3">
         <v>7899884533697</v>
@@ -13044,7 +13046,7 @@
         <v>2003066</v>
       </c>
       <c r="B568" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="C568" s="3">
         <v>7899884562796</v>
@@ -13055,7 +13057,7 @@
         <v>2003070</v>
       </c>
       <c r="B569" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="C569" s="3">
         <v>7899884563212</v>
@@ -13066,7 +13068,7 @@
         <v>1015601</v>
       </c>
       <c r="B570" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="C570" s="3">
         <v>7899884543146</v>
@@ -13077,7 +13079,7 @@
         <v>2010546</v>
       </c>
       <c r="B571" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="C571" s="3">
         <v>7899884563335</v>
@@ -13086,7 +13088,7 @@
         <v>7</v>
       </c>
       <c r="E571" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="572" spans="1:5" x14ac:dyDescent="0.25">
@@ -13094,7 +13096,7 @@
         <v>1015651</v>
       </c>
       <c r="B572" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="C572" s="3">
         <v>7899884558058</v>
@@ -13103,7 +13105,7 @@
         <v>7</v>
       </c>
       <c r="E572" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="573" spans="1:5" x14ac:dyDescent="0.25">
@@ -13111,7 +13113,7 @@
         <v>2010549</v>
       </c>
       <c r="B573" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="C573" s="3">
         <v>7899884563687</v>
@@ -13120,7 +13122,7 @@
         <v>7</v>
       </c>
       <c r="E573" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="574" spans="1:5" x14ac:dyDescent="0.25">
@@ -13128,7 +13130,7 @@
         <v>1015634</v>
       </c>
       <c r="B574" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="C574" s="3">
         <v>7899884558966</v>
@@ -13137,7 +13139,7 @@
         <v>7</v>
       </c>
       <c r="E574" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="575" spans="1:5" x14ac:dyDescent="0.25">
@@ -13145,7 +13147,7 @@
         <v>2010564</v>
       </c>
       <c r="B575" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="C575" s="3">
         <v>7899884564851</v>
@@ -13154,7 +13156,7 @@
         <v>7</v>
       </c>
       <c r="E575" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="576" spans="1:5" x14ac:dyDescent="0.25">
@@ -13162,7 +13164,7 @@
         <v>2010563</v>
       </c>
       <c r="B576" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="C576" s="3">
         <v>7899884564844</v>
@@ -13171,7 +13173,7 @@
         <v>7</v>
       </c>
       <c r="E576" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="577" spans="1:5" x14ac:dyDescent="0.25">
@@ -13179,7 +13181,7 @@
         <v>2010565</v>
       </c>
       <c r="B577" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="C577" s="3">
         <v>7899884564882</v>
@@ -13188,7 +13190,7 @@
         <v>7</v>
       </c>
       <c r="E577" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A base de reposição pode ser atualizada com inserção de produtos que não tem ainda
</commit_message>
<xml_diff>
--- a/relatorio/base.xlsx
+++ b/relatorio/base.xlsx
@@ -1,36 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Produção\Etiquetas\Nova pasta\relatorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/368431def48b862b/AGL/Automações/etiquetas/relatorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="6_{526AEF73-869F-4FAB-B2ED-062BD63BB05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-990" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -3086,6 +3071,9 @@
     <t>7899884535851</t>
   </si>
   <si>
+    <t>PINO DE DESTRAVAMENTO MANUAL PIVOTANTE EX</t>
+  </si>
+  <si>
     <t>7899884536353</t>
   </si>
   <si>
@@ -3315,15 +3303,12 @@
   </si>
   <si>
     <t>ROLAMENTO DO MANCAL DA TESTEIRA DO 200/300</t>
-  </si>
-  <si>
-    <t>PINO DE DESTRAVAMENTO MANUAL PIVOTANTE EX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3700,7 +3685,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E577"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -12319,10 +12304,10 @@
         <v>2010349</v>
       </c>
       <c r="B509" s="6" t="s">
-        <v>1090</v>
+        <v>1013</v>
       </c>
       <c r="C509" s="3" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="D509" t="s">
         <v>7</v>
@@ -12336,10 +12321,10 @@
         <v>2010495</v>
       </c>
       <c r="B510" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="C510" s="3" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="D510" t="s">
         <v>7</v>
@@ -12353,10 +12338,10 @@
         <v>2010526</v>
       </c>
       <c r="B511" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="C511" s="3" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="D511" t="s">
         <v>7</v>
@@ -12370,10 +12355,10 @@
         <v>2010373</v>
       </c>
       <c r="B512" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="C512" s="3" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="D512" t="s">
         <v>7</v>
@@ -12387,10 +12372,10 @@
         <v>2030041</v>
       </c>
       <c r="B513" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="C513" s="3" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="D513" t="s">
         <v>7</v>
@@ -12404,10 +12389,10 @@
         <v>2030050</v>
       </c>
       <c r="B514" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C514" s="3" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="D514" t="s">
         <v>7</v>
@@ -12421,10 +12406,10 @@
         <v>2001156</v>
       </c>
       <c r="B515" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="C515" s="3" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="D515" t="s">
         <v>7</v>
@@ -12438,10 +12423,10 @@
         <v>2030040</v>
       </c>
       <c r="B516" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="C516" s="3" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="D516" t="s">
         <v>7</v>
@@ -12455,10 +12440,10 @@
         <v>2030096</v>
       </c>
       <c r="B517" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="C517" s="3" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="D517" t="s">
         <v>7</v>
@@ -12472,7 +12457,7 @@
         <v>1015659</v>
       </c>
       <c r="B518" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="C518" s="3">
         <v>7899884560952</v>
@@ -12483,7 +12468,7 @@
         <v>2010372</v>
       </c>
       <c r="B519" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C519" s="3">
         <v>7899884536834</v>
@@ -12494,7 +12479,7 @@
         <v>1015613</v>
       </c>
       <c r="B520" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="C520" s="3">
         <v>7899884551905</v>
@@ -12505,7 +12490,7 @@
         <v>1015541</v>
       </c>
       <c r="B521" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="C521" s="3">
         <v>7899884527443</v>
@@ -12516,7 +12501,7 @@
         <v>1015548</v>
       </c>
       <c r="B522" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C522" s="3">
         <v>7899884531105</v>
@@ -12527,7 +12512,7 @@
         <v>1015553</v>
       </c>
       <c r="B523" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="C523" s="3">
         <v>7899884531624</v>
@@ -12536,7 +12521,7 @@
         <v>7</v>
       </c>
       <c r="E523" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="524" spans="1:5" x14ac:dyDescent="0.25">
@@ -12544,7 +12529,7 @@
         <v>1015616</v>
       </c>
       <c r="B524" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="C524" s="3">
         <v>7899884552957</v>
@@ -12555,7 +12540,7 @@
         <v>1015544</v>
       </c>
       <c r="B525" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="C525" s="3">
         <v>7899884527825</v>
@@ -12566,7 +12551,7 @@
         <v>1015543</v>
       </c>
       <c r="B526" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="C526" s="3">
         <v>7899884527818</v>
@@ -12577,7 +12562,7 @@
         <v>2030112</v>
       </c>
       <c r="B527" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="C527" s="3">
         <v>7899884562031</v>
@@ -12588,7 +12573,7 @@
         <v>1015574</v>
       </c>
       <c r="B528" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="C528" s="3">
         <v>7899884535455</v>
@@ -12610,7 +12595,7 @@
         <v>2010527</v>
       </c>
       <c r="B530" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="C530" s="3">
         <v>7899884561980</v>
@@ -12621,7 +12606,7 @@
         <v>2010528</v>
       </c>
       <c r="B531" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="C531" s="3">
         <v>7899884561997</v>
@@ -12632,7 +12617,7 @@
         <v>2010529</v>
       </c>
       <c r="B532" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="C532" s="3">
         <v>7899884562000</v>
@@ -12643,18 +12628,18 @@
         <v>2010099</v>
       </c>
       <c r="B533" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="C533" s="3">
         <v>7899884562062</v>
       </c>
     </row>
-    <row r="534" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="534" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A534" s="4">
         <v>1013510</v>
       </c>
       <c r="B534" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="C534" s="3">
         <v>7899884546000</v>
@@ -12663,7 +12648,7 @@
         <v>7</v>
       </c>
       <c r="E534" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="535" spans="1:5" x14ac:dyDescent="0.25">
@@ -12671,7 +12656,7 @@
         <v>1013507</v>
       </c>
       <c r="B535" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="C535" s="3">
         <v>7899884543955</v>
@@ -12682,7 +12667,7 @@
         <v>1110356</v>
       </c>
       <c r="B536" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="C536" s="3">
         <v>7899884533277</v>
@@ -12691,7 +12676,7 @@
         <v>258</v>
       </c>
       <c r="E536" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="537" spans="1:5" x14ac:dyDescent="0.25">
@@ -12699,7 +12684,7 @@
         <v>1015538</v>
       </c>
       <c r="B537" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="C537" s="3">
         <v>7899884527030</v>
@@ -12708,7 +12693,7 @@
         <v>258</v>
       </c>
       <c r="E537" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.25">
@@ -12716,7 +12701,7 @@
         <v>1015549</v>
       </c>
       <c r="B538" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C538" s="3">
         <v>7892562053029</v>
@@ -12725,7 +12710,7 @@
         <v>258</v>
       </c>
       <c r="E538" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="539" spans="1:5" x14ac:dyDescent="0.25">
@@ -12733,7 +12718,7 @@
         <v>2030113</v>
       </c>
       <c r="B539" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="C539" s="3">
         <v>7899884562086</v>
@@ -12744,7 +12729,7 @@
         <v>2010535</v>
       </c>
       <c r="B540" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="C540" s="3">
         <v>7899884562543</v>
@@ -12755,7 +12740,7 @@
         <v>2010534</v>
       </c>
       <c r="B541" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="C541" s="3">
         <v>7899884562536</v>
@@ -12766,18 +12751,18 @@
         <v>2010536</v>
       </c>
       <c r="B542" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C542" s="3">
         <v>7899884562550</v>
       </c>
     </row>
-    <row r="543" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="543" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A543">
         <v>2010538</v>
       </c>
       <c r="B543" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="C543" s="5">
         <v>7899884562581</v>
@@ -12799,7 +12784,7 @@
         <v>1015661</v>
       </c>
       <c r="B545" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="C545" s="3">
         <v>7899884562598</v>
@@ -12810,7 +12795,7 @@
         <v>1015537</v>
       </c>
       <c r="B546" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="C546" s="3">
         <v>7899884527023</v>
@@ -12821,7 +12806,7 @@
         <v>2010532</v>
       </c>
       <c r="B547" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="C547" s="3">
         <v>7899884562246</v>
@@ -12829,7 +12814,7 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B548" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
@@ -12837,7 +12822,7 @@
         <v>1015615</v>
       </c>
       <c r="B549" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="C549" s="3">
         <v>7899884552629</v>
@@ -12848,7 +12833,7 @@
         <v>1015555</v>
       </c>
       <c r="B550" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="C550" s="3">
         <v>7899884531648</v>
@@ -12859,7 +12844,7 @@
         <v>1015618</v>
       </c>
       <c r="B551" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="C551" s="3">
         <v>7899884552971</v>
@@ -12870,7 +12855,7 @@
         <v>2003062</v>
       </c>
       <c r="B552" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="C552" s="3">
         <v>7899884558423</v>
@@ -12881,7 +12866,7 @@
         <v>2014024</v>
       </c>
       <c r="B553" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C553" s="3">
         <v>7899884560808</v>
@@ -12892,7 +12877,7 @@
         <v>2014025</v>
       </c>
       <c r="B554" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="C554" s="3">
         <v>7899884560815</v>
@@ -12903,7 +12888,7 @@
         <v>1015032</v>
       </c>
       <c r="B555" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C555" s="3">
         <v>7899884553732</v>
@@ -12914,7 +12899,7 @@
         <v>1015559</v>
       </c>
       <c r="B556" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="C556" s="3">
         <v>7899884532089</v>
@@ -12925,7 +12910,7 @@
         <v>1015640</v>
       </c>
       <c r="B557" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="C557" s="3">
         <v>7899884559024</v>
@@ -12936,7 +12921,7 @@
         <v>1015626</v>
       </c>
       <c r="B558" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="C558" s="3">
         <v>7899884553640</v>
@@ -12947,7 +12932,7 @@
         <v>1015636</v>
       </c>
       <c r="B559" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="C559" s="3">
         <v>7899884558980</v>
@@ -12958,7 +12943,7 @@
         <v>2010454</v>
       </c>
       <c r="B560" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="C560" s="3">
         <v>7899884557303</v>
@@ -12969,7 +12954,7 @@
         <v>2004028</v>
       </c>
       <c r="B561" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="C561" s="3">
         <v>7899884534717</v>
@@ -12980,7 +12965,7 @@
         <v>1015648</v>
       </c>
       <c r="B562" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="C562" s="3">
         <v>7899884557259</v>
@@ -12991,7 +12976,7 @@
         <v>1015580</v>
       </c>
       <c r="B563" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C563" s="3">
         <v>7899884539170</v>
@@ -13002,7 +12987,7 @@
         <v>1110351</v>
       </c>
       <c r="B564" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="C564" s="3">
         <v>7899884532737</v>
@@ -13013,7 +12998,7 @@
         <v>1015662</v>
       </c>
       <c r="B565" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="C565" s="3">
         <v>7899884563397</v>
@@ -13024,7 +13009,7 @@
         <v>2010157</v>
       </c>
       <c r="B566" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="C566" s="3">
         <v>7899884563397</v>
@@ -13035,7 +13020,7 @@
         <v>1015569</v>
       </c>
       <c r="B567" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="C567" s="3">
         <v>7899884533697</v>
@@ -13046,7 +13031,7 @@
         <v>2003066</v>
       </c>
       <c r="B568" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="C568" s="3">
         <v>7899884562796</v>
@@ -13057,7 +13042,7 @@
         <v>2003070</v>
       </c>
       <c r="B569" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="C569" s="3">
         <v>7899884563212</v>
@@ -13068,7 +13053,7 @@
         <v>1015601</v>
       </c>
       <c r="B570" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="C570" s="3">
         <v>7899884543146</v>
@@ -13079,7 +13064,7 @@
         <v>2010546</v>
       </c>
       <c r="B571" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="C571" s="3">
         <v>7899884563335</v>
@@ -13088,7 +13073,7 @@
         <v>7</v>
       </c>
       <c r="E571" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="572" spans="1:5" x14ac:dyDescent="0.25">
@@ -13096,7 +13081,7 @@
         <v>1015651</v>
       </c>
       <c r="B572" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="C572" s="3">
         <v>7899884558058</v>
@@ -13105,7 +13090,7 @@
         <v>7</v>
       </c>
       <c r="E572" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="573" spans="1:5" x14ac:dyDescent="0.25">
@@ -13113,7 +13098,7 @@
         <v>2010549</v>
       </c>
       <c r="B573" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="C573" s="3">
         <v>7899884563687</v>
@@ -13122,7 +13107,7 @@
         <v>7</v>
       </c>
       <c r="E573" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="574" spans="1:5" x14ac:dyDescent="0.25">
@@ -13130,7 +13115,7 @@
         <v>1015634</v>
       </c>
       <c r="B574" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="C574" s="3">
         <v>7899884558966</v>
@@ -13139,7 +13124,7 @@
         <v>7</v>
       </c>
       <c r="E574" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="575" spans="1:5" x14ac:dyDescent="0.25">
@@ -13147,7 +13132,7 @@
         <v>2010564</v>
       </c>
       <c r="B575" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="C575" s="3">
         <v>7899884564851</v>
@@ -13156,7 +13141,7 @@
         <v>7</v>
       </c>
       <c r="E575" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="576" spans="1:5" x14ac:dyDescent="0.25">
@@ -13164,7 +13149,7 @@
         <v>2010563</v>
       </c>
       <c r="B576" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="C576" s="3">
         <v>7899884564844</v>
@@ -13173,7 +13158,7 @@
         <v>7</v>
       </c>
       <c r="E576" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="577" spans="1:5" x14ac:dyDescent="0.25">
@@ -13181,7 +13166,7 @@
         <v>2010565</v>
       </c>
       <c r="B577" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="C577" s="3">
         <v>7899884564882</v>
@@ -13190,7 +13175,7 @@
         <v>7</v>
       </c>
       <c r="E577" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>